<commit_message>
Execute Cart test cases and refine wording
</commit_message>
<xml_diff>
--- a/Test-Cases/Test-Cases-Cart.xlsx
+++ b/Test-Cases/Test-Cases-Cart.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\0. Documentos\Github\qa-saucedemo-testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38CCD4FC-C30F-4D69-B06D-886ECBBBB714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40D2409C-2E03-4C8A-88FC-698DB38EC8E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-75" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases - Cart" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -63,12 +63,6 @@
     <t>High</t>
   </si>
   <si>
-    <t>Given the user is on the inventory page
-When they add "Sauce Labs Backpack" and "Sauce Labs Bike Light" to the cart
-Then both products appear listed when entering the cart view
-And the cart icon displays the number "2"</t>
-  </si>
-  <si>
     <t>Pass</t>
   </si>
   <si>
@@ -81,12 +75,6 @@
     <t>Medium</t>
   </si>
   <si>
-    <t>Given the user has 2 products in the cart ("Sauce Labs Backpack" and "Sauce Labs Bike Light")
-When they enter the cart view
-And they click "Remove" on both products
-Then both products are successfully removed from the cart list</t>
-  </si>
-  <si>
     <t>TC-003</t>
   </si>
   <si>
@@ -96,33 +84,13 @@
     <t>Edge case / State Transition</t>
   </si>
   <si>
-    <t>Given the user has 4 products saved in the cart
-When they open the hamburger menu and click "Logout"
-And they log in again with the same credentials
-Then the 4 products are still present in the cart</t>
-  </si>
-  <si>
     <t>TC-004</t>
   </si>
   <si>
     <t>Return to inventory from the cart without losing the session</t>
   </si>
   <si>
-    <t>Both products were added successfully and appear correctly listed in the cart.</t>
-  </si>
-  <si>
     <t>Both products were removed successfully from the cart.</t>
-  </si>
-  <si>
-    <t>As expected, though possibly by design rather than a bug: cart is not cleared on logout, products persist across the logout/login transition.</t>
-  </si>
-  <si>
-    <t>Given the user has products saved in the cart
-When they return to the inventory page using the "Continue Shopping" button, or using the browser's back arrow
-Then the session remains active and the user stays logged in, with the cart items unaffected</t>
-  </si>
-  <si>
-    <t>As expected: the session remains active after returning to the inventory from the cart, using either the "Continue Shopping" button or the browser's back arrow.</t>
   </si>
   <si>
     <t>TC-005</t>
@@ -137,13 +105,46 @@
     <t>Fail</t>
   </si>
   <si>
-    <t>The system does not block or warn. It allows the user to proceed directly to the checkout form with 0 items in the cart.</t>
-  </si>
-  <si>
-    <t>Checkout is allowed with an empty cart</t>
-  </si>
-  <si>
     <t>Negative / Edge case</t>
+  </si>
+  <si>
+    <t>Given the user has 2 products in the cart ("Sauce Labs Backpack" and "Sauce Labs Bike Light")
+When they enter the cart view
+And they click "Remove" on both products
+Then both products should be successfully removed from the cart list</t>
+  </si>
+  <si>
+    <t>Given the user has 4 products saved in the cart
+When they open the hamburger menu and click "Logout"
+And they log in again with the same valid credentials
+Then the 4 products should still be present in the cart, since the user's selection is expected to be preserved between sessions</t>
+  </si>
+  <si>
+    <t>The 4 products are still present in the cart after logging back in.</t>
+  </si>
+  <si>
+    <t>Given the user is logged in with products saved in the cart
+And the user is on the cart page
+When they return to the inventory page using each of these options, one at a time: the "Continue Shopping" button and the browser's back arrow
+Then in both cases the session should remain active, the user should stay logged in, and the cart items should be unaffected</t>
+  </si>
+  <si>
+    <t>The session remains active and the cart items are unaffected when returning with the "Continue Shopping" button and with the browser's back arrow.</t>
+  </si>
+  <si>
+    <t>Given the user is on the inventory page
+When they add "Sauce Labs Backpack" and "Sauce Labs Bike Light" to the cart
+Then both products should be listed in the cart view
+And the cart icon should display the number "2"</t>
+  </si>
+  <si>
+    <t>Both products are listed in the cart and the cart icon displays "2".</t>
+  </si>
+  <si>
+    <t>Proceed to checkout with an empty cart</t>
+  </si>
+  <si>
+    <t>Then the system should not allow proceeding to checkout, and should indicate that the cart is empty</t>
   </si>
 </sst>
 </file>
@@ -241,7 +242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -261,9 +262,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -538,7 +543,7 @@
     <col min="5" max="5" width="75" customWidth="1"/>
     <col min="6" max="6" width="55" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="8" max="8" width="14" style="9" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -563,7 +568,7 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="8" t="s">
         <v>7</v>
       </c>
     </row>
@@ -581,116 +586,126 @@
         <v>11</v>
       </c>
       <c r="E2" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="2"/>
+      <c r="H2" s="7">
+        <v>46308</v>
+      </c>
     </row>
     <row r="3" spans="1:8" ht="71.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>15</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H3" s="2"/>
+        <v>12</v>
+      </c>
+      <c r="H3" s="7">
+        <v>46308</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="69.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="D4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" s="7">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="B5" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" spans="1:8" ht="67.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>23</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" s="2"/>
+        <v>12</v>
+      </c>
+      <c r="H5" s="7">
+        <v>46308</v>
+      </c>
     </row>
     <row r="6" spans="1:8" ht="79.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>33</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="H6" s="2"/>
+        <v>34</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H6" s="7">
+        <v>46308</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="G2:G5" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="G2:G6" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Pass,Fail,Blocked,Pending"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>